<commit_message>
feat: refactor NCD forms and add new screening modules with supporting media assets
</commit_message>
<xml_diff>
--- a/config/demo/forms/app/cbac_followup.xlsx
+++ b/config/demo/forms/app/cbac_followup.xlsx
@@ -383,7 +383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18.68" customWidth="1" style="6" min="1" max="1"/>
@@ -579,39 +579,46 @@
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="7">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>hidden</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>form_sync_timestamp</t>
-        </is>
-      </c>
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>inputs</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Patient &amp; CHW Info</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
+      <c r="I8" s="9" t="n"/>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="7">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>hidden</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>inputs</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Patient &amp; CHW Info</t>
-        </is>
-      </c>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n"/>
       <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
+      <c r="E9" s="9" t="n"/>
       <c r="F9" s="9" t="n"/>
       <c r="G9" s="9" t="n"/>
       <c r="H9" s="9" t="n"/>
@@ -625,7 +632,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>source_id</t>
         </is>
       </c>
       <c r="C10" s="9" t="n"/>
@@ -639,12 +646,12 @@
     <row r="11" ht="15.75" customHeight="1" s="7">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>hidden</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>source_id</t>
+          <t>user</t>
         </is>
       </c>
       <c r="C11" s="9" t="n"/>
@@ -658,12 +665,12 @@
     <row r="12" ht="15.75" customHeight="1" s="7">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>hidden</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>user</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C12" s="9" t="n"/>
@@ -682,7 +689,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="C13" s="9" t="n"/>
@@ -696,12 +703,12 @@
     <row r="14" ht="15.75" customHeight="1" s="7">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>hidden</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>user</t>
         </is>
       </c>
       <c r="C14" s="9" t="n"/>
@@ -715,12 +722,12 @@
     <row r="15" ht="15.75" customHeight="1" s="7">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>user</t>
+          <t>contact</t>
         </is>
       </c>
       <c r="C15" s="9" t="n"/>
@@ -734,21 +741,34 @@
     <row r="16" ht="15.75" customHeight="1" s="7">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>string</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>contact</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="n"/>
+          <t>_id</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Patient's Name</t>
+        </is>
+      </c>
       <c r="D16" s="9" t="n"/>
-      <c r="E16" s="9" t="n"/>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>select-contact type-person role-patient</t>
+        </is>
+      </c>
       <c r="F16" s="9" t="n"/>
       <c r="G16" s="9" t="n"/>
       <c r="H16" s="9" t="n"/>
       <c r="I16" s="9" t="n"/>
+      <c r="J16" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="7">
       <c r="A17" s="9" t="inlineStr">
@@ -758,29 +778,24 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>_id</t>
+          <t>patient_id</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Patient's Name</t>
+          <t>Medic ID</t>
         </is>
       </c>
       <c r="D17" s="9" t="n"/>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>select-contact type-person role-patient</t>
+          <t>hidden</t>
         </is>
       </c>
       <c r="F17" s="9" t="n"/>
       <c r="G17" s="9" t="n"/>
       <c r="H17" s="9" t="n"/>
       <c r="I17" s="9" t="n"/>
-      <c r="J17" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="7">
       <c r="A18" s="9" t="inlineStr">
@@ -790,12 +805,12 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>patient_id</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Medic ID</t>
+          <t>Patient Name</t>
         </is>
       </c>
       <c r="D18" s="9" t="n"/>
@@ -812,25 +827,17 @@
     <row r="19" ht="15.75" customHeight="1" s="7">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>Patient Name</t>
-        </is>
-      </c>
+          <t>contact</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="n"/>
       <c r="D19" s="9" t="n"/>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
-          <t>hidden</t>
-        </is>
-      </c>
+      <c r="E19" s="9" t="n"/>
       <c r="F19" s="9" t="n"/>
       <c r="G19" s="9" t="n"/>
       <c r="H19" s="9" t="n"/>
@@ -844,7 +851,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>inputs</t>
         </is>
       </c>
       <c r="C20" s="9" t="n"/>
@@ -856,16 +863,8 @@
       <c r="I20" s="9" t="n"/>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="7">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>end group</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>inputs</t>
-        </is>
-      </c>
+      <c r="A21" s="9" t="n"/>
+      <c r="B21" s="9" t="n"/>
       <c r="C21" s="9" t="n"/>
       <c r="D21" s="9" t="n"/>
       <c r="E21" s="9" t="n"/>
@@ -875,11 +874,23 @@
       <c r="I21" s="9" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="7">
-      <c r="A22" s="9" t="n"/>
-      <c r="B22" s="9" t="n"/>
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>ncd_followup</t>
+        </is>
+      </c>
       <c r="C22" s="9" t="n"/>
       <c r="D22" s="9" t="n"/>
-      <c r="E22" s="9" t="n"/>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="F22" s="9" t="n"/>
       <c r="G22" s="9" t="n"/>
       <c r="H22" s="9" t="n"/>
@@ -888,23 +899,27 @@
     <row r="23" ht="15.75" customHeight="1" s="7">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>ncd_followup</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="n"/>
+          <t>ncd_day_visited</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Did the patient visit for NCD day?</t>
+        </is>
+      </c>
       <c r="D23" s="9" t="n"/>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
+      <c r="E23" s="9" t="n"/>
       <c r="F23" s="9" t="n"/>
-      <c r="G23" s="9" t="n"/>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="H23" s="9" t="n"/>
       <c r="I23" s="9" t="n"/>
     </row>
@@ -916,12 +931,12 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>ncd_day_visited</t>
+          <t>willing_for_checkup</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Did the patient visit for NCD day?</t>
+          <t>Is the patient willing to go for checkup?</t>
         </is>
       </c>
       <c r="D24" s="9" t="n"/>
@@ -929,26 +944,30 @@
       <c r="F24" s="9" t="n"/>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H24" s="9" t="n"/>
+          <t>${ncd_day_visited} = 'no'</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>${ncd_day_visited} = 'no'</t>
+        </is>
+      </c>
       <c r="I24" s="9" t="n"/>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="7">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>willing_for_checkup</t>
+          <t>checkup_date</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Is the patient willing to go for checkup?</t>
+          <t>When can the patient go for checkup?</t>
         </is>
       </c>
       <c r="D25" s="9" t="n"/>
@@ -956,12 +975,12 @@
       <c r="F25" s="9" t="n"/>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>${ncd_day_visited} = 'no'</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
-          <t>${ncd_day_visited} = 'no'</t>
+          <t>${willing_for_checkup} = 'yes'</t>
         </is>
       </c>
       <c r="I25" s="9" t="n"/>
@@ -969,32 +988,24 @@
     <row r="26" ht="15.75" customHeight="1" s="7">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>checkup_date</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>When can the patient go for checkup?</t>
-        </is>
-      </c>
+          <t>t_ncd_day_visited</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="n"/>
       <c r="D26" s="9" t="n"/>
       <c r="E26" s="9" t="n"/>
-      <c r="F26" s="9" t="n"/>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H26" s="9" t="inlineStr">
-        <is>
-          <t>${willing_for_checkup} = 'yes'</t>
-        </is>
-      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>${ncd_day_visited}</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="n"/>
+      <c r="H26" s="9" t="n"/>
       <c r="I26" s="9" t="n"/>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="7">
@@ -1005,7 +1016,7 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>t_ncd_day_visited</t>
+          <t>t_willing_for_checkup</t>
         </is>
       </c>
       <c r="C27" s="9" t="n"/>
@@ -1013,7 +1024,7 @@
       <c r="E27" s="9" t="n"/>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>${ncd_day_visited}</t>
+          <t>${willing_for_checkup}</t>
         </is>
       </c>
       <c r="G27" s="9" t="n"/>
@@ -1028,7 +1039,7 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>t_willing_for_checkup</t>
+          <t>t_checkup_date</t>
         </is>
       </c>
       <c r="C28" s="9" t="n"/>
@@ -1036,7 +1047,7 @@
       <c r="E28" s="9" t="n"/>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>${willing_for_checkup}</t>
+          <t>${checkup_date}</t>
         </is>
       </c>
       <c r="G28" s="9" t="n"/>
@@ -1046,35 +1057,29 @@
     <row r="29" ht="15.75" customHeight="1" s="7">
       <c r="A29" s="9" t="inlineStr">
         <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>ncd_followup</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>t_checkup_date</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="n"/>
-      <c r="D29" s="9" t="n"/>
-      <c r="E29" s="9" t="n"/>
-      <c r="F29" s="9" t="inlineStr">
-        <is>
-          <t>${checkup_date}</t>
-        </is>
-      </c>
-      <c r="G29" s="9" t="n"/>
-      <c r="H29" s="9" t="n"/>
-      <c r="I29" s="9" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>end group</t>
-        </is>
-      </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>ncd_followup</t>
+          <t>form_submit_timestamp_iso</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>format-date-time(now(), '%Y-%m-%dT%H:%M:%S+05:30')</t>
         </is>
       </c>
     </row>
@@ -1086,27 +1091,10 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>form_submit_timestamp_iso</t>
+          <t>form_submit_timestamp_display</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>format-date-time(now(), '%Y-%m-%dT%H:%M:%S+05:30')</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>calculate</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>form_submit_timestamp_display</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>format-date-time(now(), '%e-%b-%Y %H:%M:%S')</t>
         </is>

</xml_diff>